<commit_message>
PAUT LIST OF STUDIES REDY
</commit_message>
<xml_diff>
--- a/02.FOMD/02.metadata_structure/00_FOMD_ROSES.xlsx
+++ b/02.FOMD/02.metadata_structure/00_FOMD_ROSES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-AgroecologyKnowledgeHub/Shared Documents/General/Agroecology_Evidence_Hub/02.FOMD/02.metadata_structure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{2F06371F-12C4-490E-B574-5164683F72A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3D703AA-CD71-4C29-8D6D-BF3C621E57D2}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{2F06371F-12C4-490E-B574-5164683F72A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FB48A14-BF79-4B0D-A4AF-F4A2ED0B6824}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="30060" yWindow="1815" windowWidth="21600" windowHeight="11175" xr2:uid="{83D602D3-2FE2-4AFC-A839-EADA8530BF7B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83D602D3-2FE2-4AFC-A839-EADA8530BF7B}"/>
   </bookViews>
   <sheets>
     <sheet name="00_FOMD_Roses" sheetId="1" r:id="rId1"/>
@@ -551,6 +551,9 @@
       <c r="B5">
         <v>292</v>
       </c>
+      <c r="C5">
+        <v>274</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update FOMD effect size pipeline
</commit_message>
<xml_diff>
--- a/02.FOMD/02.metadata_structure/00_FOMD_ROSES.xlsx
+++ b/02.FOMD/02.metadata_structure/00_FOMD_ROSES.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-AgroecologyKnowledgeHub/Shared Documents/General/Agroecology_Evidence_Hub/02.FOMD/02.metadata_structure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{2F06371F-12C4-490E-B574-5164683F72A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A8EA8A6-555D-4EBC-BA9D-8C1B86CDDA11}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{2F06371F-12C4-490E-B574-5164683F72A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53690C58-3BA3-420A-88F4-D1795B08471F}"/>
   <bookViews>
     <workbookView xWindow="57490" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{83D602D3-2FE2-4AFC-A839-EADA8530BF7B}"/>
   </bookViews>
   <sheets>
     <sheet name="00_FOMD_Roses" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -548,7 +548,7 @@
         <v>237</v>
       </c>
       <c r="C4">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>